<commit_message>
Professores semana 1: nomes técnicos limpos e alinhados à numeração
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AahsCeqM2DTecRKsTTfJbG
</commit_message>
<xml_diff>
--- a/kobo/professores_semana1_diagnostico.xlsx
+++ b/kobo/professores_semana1_diagnostico.xlsx
@@ -649,7 +649,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>q0_11</t>
+          <t>q0_1</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>q0_1</t>
+          <t>q0_2</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>q0_2</t>
+          <t>q0_3</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>q0_3</t>
+          <t>q0_4</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>q0_4</t>
+          <t>q0_5</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>q0_5</t>
+          <t>q0_6</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -796,7 +796,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>q0_5_outro</t>
+          <t>q0_6_outro</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>${q0_5} = 'outro'</t>
+          <t>${q0_6} = 'outro'</t>
         </is>
       </c>
     </row>
@@ -823,7 +823,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>q0_6</t>
+          <t>q0_7</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>q0_6_outro</t>
+          <t>q0_7_outro</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -860,7 +860,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>selected(${q0_6}, 'outro')</t>
+          <t>selected(${q0_7}, 'outro')</t>
         </is>
       </c>
     </row>
@@ -872,7 +872,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>q0_7</t>
+          <t>q0_8</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -894,7 +894,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>q0_8</t>
+          <t>q0_9</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -931,7 +931,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>q0_8_outro</t>
+          <t>q0_9_outro</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -946,7 +946,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>selected(${q0_8}, 'outro')</t>
+          <t>selected(${q0_9}, 'outro')</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>q0_9</t>
+          <t>q0_10</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -990,7 +990,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>q0_10</t>
+          <t>q0_11</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Q0_15_Tempo_de_atua_o_anos</t>
+          <t>q0_16</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1611,12 +1611,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>select_multiple lr9gu49</t>
+          <t>select_multiple agua_fonte</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Q1_5_Fonte_de_abastecimento_de_gua</t>
+          <t>q1_5</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>selected(${Q1_5_Fonte_de_abastecimento_de_gua}, 'outra')</t>
+          <t>selected(${q1_5}, 'outra')</t>
         </is>
       </c>
     </row>
@@ -2249,7 +2249,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>q1_23</t>
+          <t>q1_22</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2271,7 +2271,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>q1_23_outro</t>
+          <t>q1_22_outro</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2286,7 +2286,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>selected(${q1_23}, 'outro')</t>
+          <t>selected(${q1_22}, 'outro')</t>
         </is>
       </c>
     </row>
@@ -2298,7 +2298,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>q1_24</t>
+          <t>q1_23</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2320,7 +2320,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>q1_25</t>
+          <t>q1_24</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>${q1_24} = 'sim'</t>
+          <t>${q1_23} = 'sim'</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>q1_26</t>
+          <t>q1_25</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2379,7 +2379,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>q1_27</t>
+          <t>q1_26</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>${q1_26} = 'sim'</t>
+          <t>${q1_25} = 'sim'</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>q1_29</t>
+          <t>q1_27</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -2431,7 +2431,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>${q1_26} = 'sim'</t>
+          <t>${q1_25} = 'sim'</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -2448,7 +2448,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>q1_30</t>
+          <t>q1_28</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -2475,7 +2475,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>q1_31</t>
+          <t>q1_29</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -2490,7 +2490,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>${q1_30} = 'sim'</t>
+          <t>${q1_28} = 'sim'</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -2507,7 +2507,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>q1_32</t>
+          <t>q1_30</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -2522,7 +2522,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>${q1_30} = 'sim'</t>
+          <t>${q1_28} = 'sim'</t>
         </is>
       </c>
     </row>
@@ -2534,7 +2534,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>q1_33</t>
+          <t>q1_31</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -2549,7 +2549,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>${q1_30} = 'sim'</t>
+          <t>${q1_28} = 'sim'</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>q1_33_outro</t>
+          <t>q1_31_outro</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -2576,7 +2576,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>(${q1_30}='sim') and selected(${q1_33}, 'outro')</t>
+          <t>(${q1_28}='sim') and selected(${q1_31}, 'outro')</t>
         </is>
       </c>
     </row>
@@ -2588,7 +2588,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>q1_34</t>
+          <t>q1_32</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>${q1_30} = 'sim'</t>
+          <t>${q1_28} = 'sim'</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -4395,12 +4395,12 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>lr9gu49</t>
+          <t>agua_fonte</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>po_o</t>
+          <t>poco</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -4412,7 +4412,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>lr9gu49</t>
+          <t>agua_fonte</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -4429,7 +4429,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>lr9gu49</t>
+          <t>agua_fonte</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4446,12 +4446,12 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>lr9gu49</t>
+          <t>agua_fonte</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>rede_p_blica</t>
+          <t>rede_publica</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -4463,12 +4463,12 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>lr9gu49</t>
+          <t>agua_fonte</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>n_o_sabe</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -4480,7 +4480,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>lr9gu49</t>
+          <t>agua_fonte</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -5331,7 +5331,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>com_rcios</t>
+          <t>comercios</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">

</xml_diff>